<commit_message>
Replace red focus/selection styling with #C09696; widen drawer to 40vw with exit animation; global search UX fixes
Fixes a CSS cascade-layer bug where the global :focus-visible rule (left
unlayered) always beat Tailwind's layered focus-visible:/focus-within:
utilities, silently blocking every field-specific focus color override.
Migrates all form-control focus/selection states (checkboxes, radios,
selectable cards, chips) from the default red to --field-selected
(#C09696), and wires LocationInput/ContactPhoneInput into the address and
contact-edit flows they were built for. Also widens the side drawer to
40% of viewport width and gives it a slide-out close animation instead of
an instant unmount, and fixes the global search box (left-align input
text, add a clear button, stop backdrop clicks from dismissing drawers).
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/VFQ_DXP_Abbreviations_Reference.xlsx
+++ b/vfq-dxp-app/reference/VFQ_DXP_Abbreviations_Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295A2DE0-4A51-9247-A890-39555DEA6081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E09C409-A617-284A-A53A-A39AD584196F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1460" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Abbreviations" sheetId="1" r:id="rId1"/>

</xml_diff>